<commit_message>
Modificattion pour le mapping c81418a1c3e1b91a1feeaefd669366e6f8f0260c
</commit_message>
<xml_diff>
--- a/add-info-dmp/ig/StructureDefinition-ActorPS.xlsx
+++ b/add-info-dmp/ig/StructureDefinition-ActorPS.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-19T16:11:49+00:00</t>
+    <t>2025-08-01T13:09:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,9 @@
     <t>Description</t>
   </si>
   <si>
-    <t xml:space="preserve">Cet attribut représente un acteur PS. </t>
+    <t xml:space="preserve">
+Cet attribut représente un acteur PS.
+</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -231,7 +233,7 @@
     <t>Constraint(s)</t>
   </si>
   <si>
-    <t>Mapping: null</t>
+    <t>Mapping: ActorXDSCDA</t>
   </si>
   <si>
     <t/>
@@ -378,7 +380,7 @@
 </t>
   </si>
   <si>
-    <t>Type de nom : Valeur en fonction de l’auteur :  D, pour les personnes physiques, • U, pour les systèmes.</t>
+    <t>Type de nom : Valeur en fonction de l’auteur :  D, pour les personnes physiques, -U, pour les systèmes.</t>
   </si>
   <si>
     <t>D</t>

</xml_diff>

<commit_message>
chore: passage au template 2 (support i18n)
- Ajoute les paramètres i18n dans sushi-config.yaml (path-expansion-params,
  i18n-default-lang/lang, translation-sources, apply-jurisdiction, logging)
- Crée expansion-params.json (SNOMED CT + displayLanguage fr-FR)
- Crée input/pagecontent/translationinfo.md
- Crée input/translations/en/ (dossier requis pour les traductions EN)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> e440a34a78246e7af318a09cea83ea132020f7eb
</commit_message>
<xml_diff>
--- a/add-info-dmp/ig/StructureDefinition-ActorPS.xlsx
+++ b/add-info-dmp/ig/StructureDefinition-ActorPS.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-04T13:10:17+00:00</t>
+    <t>2026-06-10T15:39:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -110,7 +110,7 @@
     <t>Base Definition</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/pdsm4dmp/StructureDefinition/ActorXDS</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/pdsm4dmp/StructureDefinition/ActorXDS|0.1.0</t>
   </si>
   <si>
     <t>Abstract</t>

</xml_diff>

<commit_message>
fix: correction du libellé de jurisdiction (France (la))
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> 0e756f859c3bef3bc8a107b350003dc140addbf7
</commit_message>
<xml_diff>
--- a/add-info-dmp/ig/StructureDefinition-ActorPS.xlsx
+++ b/add-info-dmp/ig/StructureDefinition-ActorPS.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-10T15:39:40+00:00</t>
+    <t>2026-06-10T15:45:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>FRANCE</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>